<commit_message>
update new auditlog pages, fix all the currnet problem based on the new requrements
</commit_message>
<xml_diff>
--- a/samplefile.xlsx
+++ b/samplefile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb19d144c85781ad/Documents/HackSpireCode/HackSpireBE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A637266-5DA2-424D-855B-5985B0B51A7C}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F672F8E9-7DFE-4E00-B416-56DF13283FAE}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1944" yWindow="2616" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -224,6 +224,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -544,7 +548,7 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
@@ -683,6 +687,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{669EEEFE-3E12-49B5-866C-611491FA902E}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{68A35045-1DAC-4332-801D-5AF0AC4B4FCC}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add authentication through supabase, implemented forgot password under participants controls, and chnage email and reset password under admin controll, (no feature chnage email on user)
</commit_message>
<xml_diff>
--- a/samplefile.xlsx
+++ b/samplefile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb19d144c85781ad/Documents/HackSpireCode/HackSpireBE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F672F8E9-7DFE-4E00-B416-56DF13283FAE}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B478CE32-5C5C-424C-BED0-64E7C02675B1}"/>
   <bookViews>
     <workbookView xWindow="1944" yWindow="2616" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>name</t>
   </si>
@@ -43,124 +43,67 @@
     <t>preferred_role</t>
   </si>
   <si>
-    <t>Aisyah Rahman</t>
-  </si>
-  <si>
-    <t>aisyah@student.edu.my</t>
-  </si>
-  <si>
-    <t>A100001</t>
-  </si>
-  <si>
-    <t>P0001</t>
-  </si>
-  <si>
-    <t>Universiti Malaya</t>
-  </si>
-  <si>
     <t>React, Node.js</t>
   </si>
   <si>
     <t>Frontend</t>
   </si>
   <si>
-    <t>Ben Tan</t>
-  </si>
-  <si>
-    <t>ben@student.edu.my</t>
-  </si>
-  <si>
-    <t>A100002</t>
-  </si>
-  <si>
-    <t>P0002</t>
-  </si>
-  <si>
-    <t>Universiti Sains Malaysia</t>
-  </si>
-  <si>
     <t>Python</t>
   </si>
   <si>
     <t>Backend</t>
   </si>
   <si>
-    <t>Chen Wei</t>
-  </si>
-  <si>
-    <t>chen@student.edu.my</t>
-  </si>
-  <si>
-    <t>A100003</t>
-  </si>
-  <si>
-    <t>P0003</t>
-  </si>
-  <si>
-    <t>Universiti Teknologi Malaysia</t>
-  </si>
-  <si>
     <t>Figma, UI Design</t>
   </si>
   <si>
     <t>Design</t>
   </si>
   <si>
-    <t>Devi Kumar</t>
-  </si>
-  <si>
-    <t>devi@student.edu.my</t>
-  </si>
-  <si>
-    <t>A100004</t>
-  </si>
-  <si>
-    <t>P0004</t>
-  </si>
-  <si>
-    <t>Universiti Putra Malaysia</t>
-  </si>
-  <si>
-    <t>Public Speaking, Pitching</t>
-  </si>
-  <si>
-    <t>Pitching</t>
-  </si>
-  <si>
-    <t>Emir Hakim</t>
-  </si>
-  <si>
-    <t>emir@student.edu.my</t>
-  </si>
-  <si>
-    <t>A100005</t>
-  </si>
-  <si>
-    <t>P0005</t>
-  </si>
-  <si>
-    <t>Universiti Kebangsaan Malaysia</t>
-  </si>
-  <si>
-    <t>Flutter, Dart</t>
-  </si>
-  <si>
-    <t>Mobile</t>
-  </si>
-  <si>
-    <t>Farah Lim</t>
-  </si>
-  <si>
-    <t>A100006</t>
-  </si>
-  <si>
-    <t>P0006</t>
-  </si>
-  <si>
-    <t>farah@student.edu.my</t>
-  </si>
-  <si>
-    <t>P0007</t>
+    <t>mohdadlisyukri@gmail.com</t>
+  </si>
+  <si>
+    <t>peghokman@gmail.com</t>
+  </si>
+  <si>
+    <t>mohdadlisyukrinoraman@gmail.com</t>
+  </si>
+  <si>
+    <t>SW01083745</t>
+  </si>
+  <si>
+    <t>SW01083746</t>
+  </si>
+  <si>
+    <t>SW01083747</t>
+  </si>
+  <si>
+    <t>UN_001</t>
+  </si>
+  <si>
+    <t>UP_002</t>
+  </si>
+  <si>
+    <t>MU_003</t>
+  </si>
+  <si>
+    <t>Universiti Tenaga Nasional</t>
+  </si>
+  <si>
+    <t>Universiti Teknologi Petronas</t>
+  </si>
+  <si>
+    <t>Multimedia University</t>
+  </si>
+  <si>
+    <t>Adli Syukri</t>
+  </si>
+  <si>
+    <t>Naqib Mus</t>
+  </si>
+  <si>
+    <t>Fahmi</t>
   </si>
 </sst>
 </file>
@@ -515,10 +458,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -546,148 +493,78 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="G2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{669EEEFE-3E12-49B5-866C-611491FA902E}"/>
     <hyperlink ref="B2" r:id="rId2" xr:uid="{68A35045-1DAC-4332-801D-5AF0AC4B4FCC}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{6B5A139F-B26C-44A0-B3B9-439FCB436FFD}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update new feature: implement second submission with deadline, locked submission after passed deadline, update new db in submission and notification
</commit_message>
<xml_diff>
--- a/samplefile.xlsx
+++ b/samplefile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb19d144c85781ad/Documents/HackSpireCode/HackSpireBE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B478CE32-5C5C-424C-BED0-64E7C02675B1}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31F46FB6-F1E4-4EAE-ABAE-C8F8DE7CF7BF}"/>
   <bookViews>
-    <workbookView xWindow="1944" yWindow="2616" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>name</t>
   </si>
@@ -104,6 +104,21 @@
   </si>
   <si>
     <t>Fahmi</t>
+  </si>
+  <si>
+    <t>ex</t>
+  </si>
+  <si>
+    <t>luminahackspire@gmail.com</t>
+  </si>
+  <si>
+    <t>sww</t>
+  </si>
+  <si>
+    <t>we</t>
+  </si>
+  <si>
+    <t>w</t>
   </si>
 </sst>
 </file>
@@ -458,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -466,6 +481,8 @@
     <col min="3" max="3" width="14.88671875" customWidth="1"/>
     <col min="4" max="4" width="16.77734375" customWidth="1"/>
     <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -558,6 +575,29 @@
       </c>
       <c r="G4" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -565,6 +605,7 @@
     <hyperlink ref="B3" r:id="rId1" xr:uid="{669EEEFE-3E12-49B5-866C-611491FA902E}"/>
     <hyperlink ref="B2" r:id="rId2" xr:uid="{68A35045-1DAC-4332-801D-5AF0AC4B4FCC}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{6B5A139F-B26C-44A0-B3B9-439FCB436FFD}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{1320C083-75CA-4916-85D9-783F6C7F5786}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update annpuncemnt being trigerred whenever the finalists is being published
</commit_message>
<xml_diff>
--- a/samplefile.xlsx
+++ b/samplefile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb19d144c85781ad/Documents/HackSpireCode/HackSpireBE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31F46FB6-F1E4-4EAE-ABAE-C8F8DE7CF7BF}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="11_2B59C09755FAD2547D63DCF050C1E8335181F576" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B3A3580-2AF0-4808-8000-F57F4FF80104}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2292" yWindow="2964" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>name</t>
   </si>
@@ -119,6 +119,24 @@
   </si>
   <si>
     <t>w</t>
+  </si>
+  <si>
+    <t>nips</t>
+  </si>
+  <si>
+    <t>nickdanish.hack10@gmail.com</t>
+  </si>
+  <si>
+    <t>sw</t>
+  </si>
+  <si>
+    <t>ws</t>
+  </si>
+  <si>
+    <t>Uniten</t>
+  </si>
+  <si>
+    <t>Gooners</t>
   </si>
 </sst>
 </file>
@@ -473,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -600,12 +618,36 @@
         <v>31</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{669EEEFE-3E12-49B5-866C-611491FA902E}"/>
     <hyperlink ref="B2" r:id="rId2" xr:uid="{68A35045-1DAC-4332-801D-5AF0AC4B4FCC}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{6B5A139F-B26C-44A0-B3B9-439FCB436FFD}"/>
     <hyperlink ref="B5" r:id="rId4" xr:uid="{1320C083-75CA-4916-85D9-783F6C7F5786}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{07D5DDB2-FC87-4FC8-9610-378763217441}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>